<commit_message>
Integrate AVERAGE and COUNT into the ranges section
The section is now "Ranges and Functions" and introduces SUM, AVERAGE and
COUNT together as functions that take a range, rather than treating the latter
two as a subsection. The workbook gains average and count rows.

AVERAGE is applied to acres and bushels only -- averaging the yield column is
left for Module 1c, where weighted averages are explained, and the chapter now
says so instead of alluding to the IF functions.

Also corrects module01c's weighted-average example, which described nine barley
varieties at B2:B10 that this workbook never contained.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_conditional_practice.xlsx
+++ b/textbook_examples/mod01_conditional_practice.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Conditional" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -29,35 +28,41 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="004A7C59"/>
+      <color rgb="FF4A7C59"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="005C6B62"/>
+      <family val="2"/>
+      <color rgb="FF5C6B62"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="0024302A"/>
+      <family val="2"/>
+      <color rgb="FF24302A"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Consolas"/>
-      <color rgb="002F5D46"/>
+      <family val="2"/>
+      <color rgb="FF2F5D46"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="0024302A"/>
+      <color rgb="FF24302A"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -70,7 +75,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004A7C59"/>
+        <fgColor rgb="FF4A7C59"/>
       </patternFill>
     </fill>
   </fills>
@@ -86,12 +91,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
@@ -110,10 +112,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -477,280 +484,280 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" style="11" min="1" max="1"/>
+    <col width="15" customWidth="1" style="11" min="2" max="2"/>
+    <col width="11" customWidth="1" style="11" min="3" max="3"/>
+    <col width="13" customWidth="1" style="11" min="4" max="4"/>
+    <col width="11" customWidth="1" style="11" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1">
+    <row r="1" ht="18" customHeight="1" s="11">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Conditional functions</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="44" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="44" customHeight="1" s="11">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Eight fields, each with a crop and a yield.  The functions below all answer questions about a SUBSET of the rows — only the canola fields, only the yields above a threshold.  Column F shows the formula that produced column E.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1"/>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="3" ht="18" customHeight="1" s="11"/>
+    <row r="4" ht="18" customHeight="1" s="11">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Crop</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Acres</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Yield (bu/ac)</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Above 50?</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="5" ht="18" customHeight="1" s="11">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>North</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Canola</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="6" t="n">
         <v>320</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="7" t="n">
         <v>41.2</v>
       </c>
-      <c r="E5" s="6" t="n"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="E5" s="5" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="11">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>South</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Wheat</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="6" t="n">
         <v>250</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="7" t="n">
         <v>58.6</v>
       </c>
-      <c r="E6" s="6" t="n"/>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="E6" s="5" t="n"/>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="11">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Creek</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Canola</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="7" t="n">
         <v>37.9</v>
       </c>
-      <c r="E7" s="6" t="n"/>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="E7" s="5" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="11">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Barley</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="7" t="n">
         <v>72.40000000000001</v>
       </c>
-      <c r="E8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="E8" s="5" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="11">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Rented</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Wheat</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="7" t="n">
         <v>61.3</v>
       </c>
-      <c r="E9" s="6" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="E9" s="5" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="11">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Airport</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Canola</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="7" t="n">
         <v>44.8</v>
       </c>
-      <c r="E10" s="6" t="n"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="E10" s="5" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Hill</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Barley</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="6" t="n">
         <v>275</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="7" t="n">
         <v>68.09999999999999</v>
       </c>
-      <c r="E11" s="6" t="n"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="E11" s="5" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="11">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Slough</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Wheat</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="6" t="n">
         <v>330</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="7" t="n">
         <v>55.2</v>
       </c>
-      <c r="E12" s="6" t="n"/>
-    </row>
-    <row r="13" ht="18" customHeight="1"/>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="E12" s="5" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="11"/>
+    <row r="14" ht="18" customHeight="1" s="11">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Questions about a subset</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="15" ht="18" customHeight="1" s="11">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>How many canola fields?</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="9" t="n"/>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="12" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="11">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Total canola acres</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="9" t="n"/>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="12" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="11">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Average canola yield</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="9" t="n"/>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="12" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="11">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>How many yields above 60?</t>
         </is>
       </c>
-      <c r="B18" s="8" t="n"/>
-      <c r="C18" s="9" t="n"/>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="12" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="11">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Average wheat yield over 250 ac</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="9" t="n"/>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="12" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="11">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>How many above the average?</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="9" t="n"/>
-    </row>
-    <row r="21" ht="18" customHeight="1"/>
-    <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="12" t="n"/>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="11"/>
+    <row r="22" ht="32" customHeight="1" s="11">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>The last one is the awkward case: the threshold is itself a calculation, so you glue "&gt;" onto it with &amp;.  Quoting the whole thing as "&gt;AVERAGE(...)" would search for that literal text.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1"/>
+    <row r="23" ht="18" customHeight="1" s="11"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A2:F2"/>

</xml_diff>